<commit_message>
throw error if plate reader channel is not valid
even if it isn't used
also fixed all tests to comply with this
</commit_message>
<xml_diff>
--- a/test/inputs/kw_name_collision.xlsx
+++ b/test/inputs/kw_name_collision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/Longwing/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A66A21A-BCA9-FF4C-ADBC-640D8AAD88C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7FEF7B-871B-7A4F-82D0-179793BC2F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>Plate</t>
   </si>
@@ -118,6 +118,30 @@
   </si>
   <si>
     <t>doubling_time(plate_01_a1, plate_01_time, Endpoints(start_time = start_time, end_time = end_time))</t>
+  </si>
+  <si>
+    <t>535_485</t>
+  </si>
+  <si>
+    <t>flu</t>
+  </si>
+  <si>
+    <t>530_485_1</t>
+  </si>
+  <si>
+    <t>flu1</t>
+  </si>
+  <si>
+    <t>530_485_2</t>
+  </si>
+  <si>
+    <t>flu2</t>
+  </si>
+  <si>
+    <t>530_485_3</t>
+  </si>
+  <si>
+    <t>flu3</t>
   </si>
 </sst>
 </file>
@@ -581,7 +605,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DA707B9-0BE9-45E5-A5EE-A3873F0594F1}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -609,6 +633,38 @@
       </c>
       <c r="B3" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>